<commit_message>
Update Invenio records (2026-06-23)
</commit_message>
<xml_diff>
--- a/data/2026-06-23_invenio-records.xlsx
+++ b/data/2026-06-23_invenio-records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
           <t>ARCURL</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -489,6 +494,11 @@
           <t>https://git.nfdi4plants.org/projects/4018/</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +536,11 @@
           <t>https://git.nfdi4plants.org/projects/810/</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -563,6 +578,11 @@
           <t>https://git.nfdi4plants.org/projects/4099/</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -600,6 +620,11 @@
           <t>https://git.nfdi4plants.org/projects/3837/</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -637,6 +662,11 @@
           <t>https://git.nfdi4plants.org/projects/3953/</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -674,6 +704,11 @@
           <t>https://git.nfdi4plants.org/projects/3932/</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -711,6 +746,11 @@
           <t>https://git.nfdi4plants.org/projects/4006/</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -748,6 +788,11 @@
           <t>https://git.nfdi4plants.org/projects/3166/</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -785,6 +830,11 @@
           <t>https://git.nfdi4plants.org/projects/3984/</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -822,6 +872,11 @@
           <t>https://git.nfdi4plants.org/projects/3861/</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -859,6 +914,11 @@
           <t>https://git.nfdi4plants.org/projects/3879/</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -896,6 +956,11 @@
           <t>https://git.nfdi4plants.org/projects/3831/</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -933,6 +998,11 @@
           <t>https://git.nfdi4plants.org/projects/3578/</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -970,6 +1040,11 @@
           <t>https://git.nfdi4plants.org/projects/3507/</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1007,6 +1082,11 @@
           <t>https://git.nfdi4plants.org/projects/3617/</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1044,6 +1124,11 @@
           <t>https://git.nfdi4plants.org/projects/3773/</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1081,6 +1166,11 @@
           <t>https://git.nfdi4plants.org/projects/3215</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1118,6 +1208,11 @@
           <t>https://git.nfdi4plants.org/projects/3048/</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1155,6 +1250,11 @@
           <t>https://git.nfdi4plants.org/projects/3444</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1192,6 +1292,11 @@
           <t>https://git.nfdi4plants.org/projects/2480</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1229,6 +1334,11 @@
           <t>https://git.nfdi4plants.org/projects/1582</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1266,6 +1376,11 @@
           <t>https://git.nfdi4plants.org/projects/3204</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1303,6 +1418,11 @@
           <t>https://git.nfdi4plants.org/projects/2792</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1340,6 +1460,11 @@
           <t>https://git.nfdi4plants.org/projects/3371/</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1377,6 +1502,11 @@
           <t>https://git.nfdi4plants.org/projects/2342</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1414,6 +1544,11 @@
           <t>https://git.nfdi4plants.org/projects/1636/</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1451,6 +1586,11 @@
           <t>https://git.nfdi4plants.org/projects/3272/</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1488,6 +1628,11 @@
           <t>https://git.nfdi4plants.org/projects/1600/</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1525,6 +1670,11 @@
           <t>https://git.nfdi4plants.org/projects/2748/</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1562,6 +1712,11 @@
           <t>https://git.nfdi4plants.org/projects/781/</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1599,6 +1754,11 @@
           <t>https://git.nfdi4plants.org/projects/3205</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1636,6 +1796,11 @@
           <t>https://git.nfdi4plants.org/projects/3172</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1673,6 +1838,11 @@
           <t>https://git.nfdi4plants.org/projects/3122</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1710,6 +1880,11 @@
           <t>https://git.nfdi4plants.org/projects/2876</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1747,6 +1922,11 @@
           <t>https://git.nfdi4plants.org/projects/2949</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1784,6 +1964,11 @@
           <t>https://git.nfdi4plants.org/projects/2886</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1821,6 +2006,11 @@
           <t>https://git.nfdi4plants.org/projects/3011</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1858,6 +2048,11 @@
           <t>https://git.nfdi4plants.org/projects/2262</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1895,6 +2090,11 @@
           <t>https://git.nfdi4plants.org/projects/3046</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1932,6 +2132,11 @@
           <t>https://git.nfdi4plants.org/projects/2948</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1969,6 +2174,11 @@
           <t>https://git.nfdi4plants.org/projects/2974</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2006,6 +2216,11 @@
           <t>https://git.nfdi4plants.org/projects/2517</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>MibiNet; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2043,6 +2258,11 @@
           <t>https://git.nfdi4plants.org/projects/2495</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2080,6 +2300,11 @@
           <t>https://git.nfdi4plants.org/projects/1590</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2117,6 +2342,11 @@
           <t>https://git.nfdi4plants.org/projects/1488</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2154,6 +2384,11 @@
           <t>https://git.nfdi4plants.org/projects/969</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2191,6 +2426,11 @@
           <t>https://git.nfdi4plants.org/projects/2188</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2228,6 +2468,11 @@
           <t>https://git.nfdi4plants.org/projects/487</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2265,6 +2510,11 @@
           <t>https://git.nfdi4plants.org/projects/1455</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>DataPLANT; CEPLAS</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2302,6 +2552,11 @@
           <t>https://git.nfdi4plants.org/projects/1399</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2339,6 +2594,11 @@
           <t>https://git.nfdi4plants.org/projects/720</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2376,6 +2636,11 @@
           <t>https://git.nfdi4plants.org/projects/719</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>MAdLand; DataPLANT</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2411,6 +2676,11 @@
       <c r="G54" t="inlineStr">
         <is>
           <t>https://git.nfdi4plants.org/projects/122</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>DataPLANT</t>
         </is>
       </c>
     </row>

</xml_diff>